<commit_message>
fixes to excel workbooks
</commit_message>
<xml_diff>
--- a/SignalStack_CashFlowCompass.xlsx
+++ b/SignalStack_CashFlowCompass.xlsx
@@ -232,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -390,6 +390,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="6" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -952,24 +958,22 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="42" t="inlineStr">
-        <is>
-          <t>10/07/2024</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="n">
+      <c r="A10" s="42" t="n">
+        <v>45572</v>
+      </c>
+      <c r="B10" s="55" t="n">
         <v>38200</v>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="55" t="n">
         <v>14200</v>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="55" t="n">
         <v>10800</v>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="55" t="n">
         <v>17500</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="55" t="n">
         <v>13200</v>
       </c>
       <c r="G10" s="11">
@@ -982,24 +986,22 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="42" t="inlineStr">
-        <is>
-          <t>10/14/2024</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="n">
+      <c r="A11" s="42" t="n">
+        <v>45579</v>
+      </c>
+      <c r="B11" s="55" t="n">
         <v>42500</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="55" t="n">
         <v>15800</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="55" t="n">
         <v>11200</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="55" t="n">
         <v>18200</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="55" t="n">
         <v>14100</v>
       </c>
       <c r="G11" s="11">
@@ -1012,24 +1014,22 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="42" t="inlineStr">
-        <is>
-          <t>10/21/2024</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="n">
+      <c r="A12" s="42" t="n">
+        <v>45586</v>
+      </c>
+      <c r="B12" s="55" t="n">
         <v>46600</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="C12" s="55" t="n">
         <v>13900</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="55" t="n">
         <v>12400</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="55" t="n">
         <v>16800</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="55" t="n">
         <v>13600</v>
       </c>
       <c r="G12" s="11">
@@ -1042,24 +1042,22 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="42" t="inlineStr">
-        <is>
-          <t>10/28/2024</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="n">
+      <c r="A13" s="42" t="n">
+        <v>45593</v>
+      </c>
+      <c r="B13" s="55" t="n">
         <v>49800</v>
       </c>
-      <c r="C13" s="11" t="n">
+      <c r="C13" s="55" t="n">
         <v>16200</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="55" t="n">
         <v>13800</v>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="55" t="n">
         <v>19100</v>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F13" s="55" t="n">
         <v>14900</v>
       </c>
       <c r="G13" s="11">
@@ -1072,24 +1070,22 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="42" t="inlineStr">
-        <is>
-          <t>11/04/2024</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="n">
+      <c r="A14" s="42" t="n">
+        <v>45600</v>
+      </c>
+      <c r="B14" s="55" t="n">
         <v>54000</v>
       </c>
-      <c r="C14" s="11" t="n">
+      <c r="C14" s="55" t="n">
         <v>14800</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="55" t="n">
         <v>11600</v>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="55" t="n">
         <v>17400</v>
       </c>
-      <c r="F14" s="11" t="n">
+      <c r="F14" s="55" t="n">
         <v>13100</v>
       </c>
       <c r="G14" s="11">
@@ -1102,24 +1098,22 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="42" t="inlineStr">
-        <is>
-          <t>11/11/2024</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="n">
+      <c r="A15" s="42" t="n">
+        <v>45607</v>
+      </c>
+      <c r="B15" s="55" t="n">
         <v>58300</v>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="55" t="n">
         <v>15100</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="55" t="n">
         <v>12200</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="55" t="n">
         <v>18000</v>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="F15" s="55" t="n">
         <v>13800</v>
       </c>
       <c r="G15" s="11">
@@ -1132,24 +1126,22 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="42" t="inlineStr">
-        <is>
-          <t>11/18/2024</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="n">
+      <c r="A16" s="42" t="n">
+        <v>45614</v>
+      </c>
+      <c r="B16" s="55" t="n">
         <v>62500</v>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C16" s="55" t="n">
         <v>13600</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="55" t="n">
         <v>14400</v>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="55" t="n">
         <v>16500</v>
       </c>
-      <c r="F16" s="11" t="n">
+      <c r="F16" s="55" t="n">
         <v>15200</v>
       </c>
       <c r="G16" s="11">
@@ -1162,24 +1154,22 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="42" t="inlineStr">
-        <is>
-          <t>11/25/2024</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="n">
+      <c r="A17" s="42" t="n">
+        <v>45621</v>
+      </c>
+      <c r="B17" s="55" t="n">
         <v>63800</v>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="C17" s="55" t="n">
         <v>12400</v>
       </c>
-      <c r="D17" s="11" t="n">
+      <c r="D17" s="55" t="n">
         <v>10800</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="55" t="n">
         <v>15800</v>
       </c>
-      <c r="F17" s="11" t="n">
+      <c r="F17" s="55" t="n">
         <v>12400</v>
       </c>
       <c r="G17" s="11">
@@ -1192,24 +1182,22 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="43" t="inlineStr">
-        <is>
-          <t>12/02/2024</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="n">
+      <c r="A18" s="43" t="n">
+        <v>45628</v>
+      </c>
+      <c r="B18" s="56" t="n">
         <v>67200</v>
       </c>
-      <c r="C18" s="14" t="n">
+      <c r="C18" s="56" t="n">
         <v>11800</v>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D18" s="56" t="n">
         <v>12600</v>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="E18" s="56" t="n">
         <v>14900</v>
       </c>
-      <c r="F18" s="14" t="n">
+      <c r="F18" s="56" t="n">
         <v>13500</v>
       </c>
       <c r="G18" s="14">
@@ -1222,24 +1210,22 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="43" t="inlineStr">
-        <is>
-          <t>12/09/2024</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="n">
+      <c r="A19" s="43" t="n">
+        <v>45635</v>
+      </c>
+      <c r="B19" s="56" t="n">
         <v>68600</v>
       </c>
-      <c r="C19" s="14" t="n">
+      <c r="C19" s="56" t="n">
         <v>13200</v>
       </c>
-      <c r="D19" s="14" t="n">
+      <c r="D19" s="56" t="n">
         <v>11400</v>
       </c>
-      <c r="E19" s="14" t="n">
+      <c r="E19" s="56" t="n">
         <v>16100</v>
       </c>
-      <c r="F19" s="14" t="n">
+      <c r="F19" s="56" t="n">
         <v>13000</v>
       </c>
       <c r="G19" s="14">
@@ -1252,24 +1238,22 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="43" t="inlineStr">
-        <is>
-          <t>12/16/2024</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="n">
+      <c r="A20" s="43" t="n">
+        <v>45642</v>
+      </c>
+      <c r="B20" s="56" t="n">
         <v>71700</v>
       </c>
-      <c r="C20" s="14" t="n">
+      <c r="C20" s="56" t="n">
         <v>9800</v>
       </c>
-      <c r="D20" s="14" t="n">
+      <c r="D20" s="56" t="n">
         <v>8400</v>
       </c>
-      <c r="E20" s="14" t="n">
+      <c r="E20" s="56" t="n">
         <v>13200</v>
       </c>
-      <c r="F20" s="14" t="n">
+      <c r="F20" s="56" t="n">
         <v>10800</v>
       </c>
       <c r="G20" s="14">
@@ -1282,24 +1266,22 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="43" t="inlineStr">
-        <is>
-          <t>12/23/2024</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="n">
+      <c r="A21" s="43" t="n">
+        <v>45649</v>
+      </c>
+      <c r="B21" s="56" t="n">
         <v>74100</v>
       </c>
-      <c r="C21" s="14" t="n">
+      <c r="C21" s="56" t="n">
         <v>6200</v>
       </c>
-      <c r="D21" s="14" t="n">
+      <c r="D21" s="56" t="n">
         <v>5600</v>
       </c>
-      <c r="E21" s="14" t="n">
+      <c r="E21" s="56" t="n">
         <v>9400</v>
       </c>
-      <c r="F21" s="14" t="n">
+      <c r="F21" s="56" t="n">
         <v>7800</v>
       </c>
       <c r="G21" s="14">
@@ -1312,24 +1294,22 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="43" t="inlineStr">
-        <is>
-          <t>12/30/2024</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="n">
+      <c r="A22" s="43" t="n">
+        <v>45656</v>
+      </c>
+      <c r="B22" s="56" t="n">
         <v>75700</v>
       </c>
-      <c r="C22" s="14" t="n">
+      <c r="C22" s="56" t="n">
         <v>5100</v>
       </c>
-      <c r="D22" s="14" t="n">
+      <c r="D22" s="56" t="n">
         <v>4800</v>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="E22" s="56" t="n">
         <v>8200</v>
       </c>
-      <c r="F22" s="14" t="n">
+      <c r="F22" s="56" t="n">
         <v>6900</v>
       </c>
       <c r="G22" s="14">
@@ -1342,24 +1322,22 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="43" t="inlineStr">
-        <is>
-          <t>01/06/2025</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="n">
+      <c r="A23" s="43" t="n">
+        <v>45663</v>
+      </c>
+      <c r="B23" s="56" t="n">
         <v>77000</v>
       </c>
-      <c r="C23" s="14" t="n">
+      <c r="C23" s="56" t="n">
         <v>14400</v>
       </c>
-      <c r="D23" s="14" t="n">
+      <c r="D23" s="56" t="n">
         <v>11800</v>
       </c>
-      <c r="E23" s="14" t="n">
+      <c r="E23" s="56" t="n">
         <v>17200</v>
       </c>
-      <c r="F23" s="14" t="n">
+      <c r="F23" s="56" t="n">
         <v>13400</v>
       </c>
       <c r="G23" s="14">
@@ -1372,24 +1350,22 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="43" t="inlineStr">
-        <is>
-          <t>01/13/2025</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="n">
+      <c r="A24" s="43" t="n">
+        <v>45670</v>
+      </c>
+      <c r="B24" s="56" t="n">
         <v>80800</v>
       </c>
-      <c r="C24" s="14" t="n">
+      <c r="C24" s="56" t="n">
         <v>15200</v>
       </c>
-      <c r="D24" s="14" t="n">
+      <c r="D24" s="56" t="n">
         <v>12600</v>
       </c>
-      <c r="E24" s="14" t="n">
+      <c r="E24" s="56" t="n">
         <v>18400</v>
       </c>
-      <c r="F24" s="14" t="n">
+      <c r="F24" s="56" t="n">
         <v>14200</v>
       </c>
       <c r="G24" s="14">
@@ -1402,24 +1378,22 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="43" t="inlineStr">
-        <is>
-          <t>01/20/2025</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="n">
+      <c r="A25" s="43" t="n">
+        <v>45677</v>
+      </c>
+      <c r="B25" s="56" t="n">
         <v>85000</v>
       </c>
-      <c r="C25" s="14" t="n">
+      <c r="C25" s="56" t="n">
         <v>14800</v>
       </c>
-      <c r="D25" s="14" t="n">
+      <c r="D25" s="56" t="n">
         <v>13200</v>
       </c>
-      <c r="E25" s="14" t="n">
+      <c r="E25" s="56" t="n">
         <v>17800</v>
       </c>
-      <c r="F25" s="14" t="n">
+      <c r="F25" s="56" t="n">
         <v>14600</v>
       </c>
       <c r="G25" s="14">
@@ -1432,24 +1406,22 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="43" t="inlineStr">
-        <is>
-          <t>01/27/2025</t>
-        </is>
-      </c>
-      <c r="B26" s="14" t="n">
+      <c r="A26" s="43" t="n">
+        <v>45684</v>
+      </c>
+      <c r="B26" s="56" t="n">
         <v>88200</v>
       </c>
-      <c r="C26" s="14" t="n">
+      <c r="C26" s="56" t="n">
         <v>16100</v>
       </c>
-      <c r="D26" s="14" t="n">
+      <c r="D26" s="56" t="n">
         <v>12400</v>
       </c>
-      <c r="E26" s="14" t="n">
+      <c r="E26" s="56" t="n">
         <v>19200</v>
       </c>
-      <c r="F26" s="14" t="n">
+      <c r="F26" s="56" t="n">
         <v>13800</v>
       </c>
       <c r="G26" s="14">
@@ -1462,24 +1434,22 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="43" t="inlineStr">
-        <is>
-          <t>02/03/2025</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="n">
+      <c r="A27" s="43" t="n">
+        <v>45691</v>
+      </c>
+      <c r="B27" s="56" t="n">
         <v>93600</v>
       </c>
-      <c r="C27" s="14" t="n">
+      <c r="C27" s="56" t="n">
         <v>15400</v>
       </c>
-      <c r="D27" s="14" t="n">
+      <c r="D27" s="56" t="n">
         <v>13800</v>
       </c>
-      <c r="E27" s="14" t="n">
+      <c r="E27" s="56" t="n">
         <v>18600</v>
       </c>
-      <c r="F27" s="14" t="n">
+      <c r="F27" s="56" t="n">
         <v>14900</v>
       </c>
       <c r="G27" s="14">
@@ -1492,24 +1462,22 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="43" t="inlineStr">
-        <is>
-          <t>02/10/2025</t>
-        </is>
-      </c>
-      <c r="B28" s="14" t="n">
+      <c r="A28" s="43" t="n">
+        <v>45698</v>
+      </c>
+      <c r="B28" s="56" t="n">
         <v>97300</v>
       </c>
-      <c r="C28" s="14" t="n">
+      <c r="C28" s="56" t="n">
         <v>14200</v>
       </c>
-      <c r="D28" s="14" t="n">
+      <c r="D28" s="56" t="n">
         <v>12200</v>
       </c>
-      <c r="E28" s="14" t="n">
+      <c r="E28" s="56" t="n">
         <v>17100</v>
       </c>
-      <c r="F28" s="14" t="n">
+      <c r="F28" s="56" t="n">
         <v>13600</v>
       </c>
       <c r="G28" s="14">
@@ -1522,24 +1490,22 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="43" t="inlineStr">
-        <is>
-          <t>02/17/2025</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="n">
+      <c r="A29" s="43" t="n">
+        <v>45705</v>
+      </c>
+      <c r="B29" s="56" t="n">
         <v>100800</v>
       </c>
-      <c r="C29" s="14" t="n">
+      <c r="C29" s="56" t="n">
         <v>15800</v>
       </c>
-      <c r="D29" s="14" t="n">
+      <c r="D29" s="56" t="n">
         <v>14100</v>
       </c>
-      <c r="E29" s="14" t="n">
+      <c r="E29" s="56" t="n">
         <v>19000</v>
       </c>
-      <c r="F29" s="14" t="n">
+      <c r="F29" s="56" t="n">
         <v>15200</v>
       </c>
       <c r="G29" s="14">
@@ -1552,24 +1518,22 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="43" t="inlineStr">
-        <is>
-          <t>02/24/2025</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="n">
+      <c r="A30" s="43" t="n">
+        <v>45712</v>
+      </c>
+      <c r="B30" s="56" t="n">
         <v>104600</v>
       </c>
-      <c r="C30" s="14" t="n">
+      <c r="C30" s="56" t="n">
         <v>14228</v>
       </c>
-      <c r="D30" s="14" t="n">
+      <c r="D30" s="56" t="n">
         <v>10515</v>
       </c>
-      <c r="E30" s="14" t="n">
+      <c r="E30" s="56" t="n">
         <v>16832</v>
       </c>
-      <c r="F30" s="14" t="n">
+      <c r="F30" s="56" t="n">
         <v>12898</v>
       </c>
       <c r="G30" s="14">
@@ -1582,24 +1546,22 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="43" t="inlineStr">
-        <is>
-          <t>03/03/2025</t>
-        </is>
-      </c>
-      <c r="B31" s="14" t="n">
+      <c r="A31" s="43" t="n">
+        <v>45719</v>
+      </c>
+      <c r="B31" s="56" t="n">
         <v>108534</v>
       </c>
-      <c r="C31" s="14" t="n">
+      <c r="C31" s="56" t="n">
         <v>16898</v>
       </c>
-      <c r="D31" s="14" t="n">
+      <c r="D31" s="56" t="n">
         <v>10443</v>
       </c>
-      <c r="E31" s="14" t="n">
+      <c r="E31" s="56" t="n">
         <v>19349</v>
       </c>
-      <c r="F31" s="14" t="n">
+      <c r="F31" s="56" t="n">
         <v>13540</v>
       </c>
       <c r="G31" s="14">
@@ -1612,24 +1574,22 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="43" t="inlineStr">
-        <is>
-          <t>03/10/2025</t>
-        </is>
-      </c>
-      <c r="B32" s="14" t="n">
+      <c r="A32" s="43" t="n">
+        <v>45726</v>
+      </c>
+      <c r="B32" s="56" t="n">
         <v>114343</v>
       </c>
-      <c r="C32" s="14" t="n">
+      <c r="C32" s="56" t="n">
         <v>13812</v>
       </c>
-      <c r="D32" s="14" t="n">
+      <c r="D32" s="56" t="n">
         <v>12129</v>
       </c>
-      <c r="E32" s="14" t="n">
+      <c r="E32" s="56" t="n">
         <v>17349</v>
       </c>
-      <c r="F32" s="14" t="n">
+      <c r="F32" s="56" t="n">
         <v>14488</v>
       </c>
       <c r="G32" s="14">
@@ -1642,24 +1602,22 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="43" t="inlineStr">
-        <is>
-          <t>03/17/2025</t>
-        </is>
-      </c>
-      <c r="B33" s="14" t="n">
+      <c r="A33" s="43" t="n">
+        <v>45733</v>
+      </c>
+      <c r="B33" s="56" t="n">
         <v>117204</v>
       </c>
-      <c r="C33" s="14" t="n">
+      <c r="C33" s="56" t="n">
         <v>15833</v>
       </c>
-      <c r="D33" s="14" t="n">
+      <c r="D33" s="56" t="n">
         <v>11949</v>
       </c>
-      <c r="E33" s="14" t="n">
+      <c r="E33" s="56" t="n">
         <v>18707</v>
       </c>
-      <c r="F33" s="14" t="n">
+      <c r="F33" s="56" t="n">
         <v>13792</v>
       </c>
       <c r="G33" s="14">
@@ -1672,24 +1630,22 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="43" t="inlineStr">
-        <is>
-          <t>03/24/2025</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="n">
+      <c r="A34" s="43" t="n">
+        <v>45740</v>
+      </c>
+      <c r="B34" s="56" t="n">
         <v>122119</v>
       </c>
-      <c r="C34" s="14" t="n">
+      <c r="C34" s="56" t="n">
         <v>14478</v>
       </c>
-      <c r="D34" s="14" t="n">
+      <c r="D34" s="56" t="n">
         <v>11303</v>
       </c>
-      <c r="E34" s="14" t="n">
+      <c r="E34" s="56" t="n">
         <v>17220</v>
       </c>
-      <c r="F34" s="14" t="n">
+      <c r="F34" s="56" t="n">
         <v>13796</v>
       </c>
       <c r="G34" s="14">
@@ -1702,24 +1658,22 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="43" t="inlineStr">
-        <is>
-          <t>03/31/2025</t>
-        </is>
-      </c>
-      <c r="B35" s="14" t="n">
+      <c r="A35" s="43" t="n">
+        <v>45747</v>
+      </c>
+      <c r="B35" s="56" t="n">
         <v>125543</v>
       </c>
-      <c r="C35" s="14" t="n">
+      <c r="C35" s="56" t="n">
         <v>16207</v>
       </c>
-      <c r="D35" s="14" t="n">
+      <c r="D35" s="56" t="n">
         <v>12220</v>
       </c>
-      <c r="E35" s="14" t="n">
+      <c r="E35" s="56" t="n">
         <v>18837</v>
       </c>
-      <c r="F35" s="14" t="n">
+      <c r="F35" s="56" t="n">
         <v>13628</v>
       </c>
       <c r="G35" s="14">
@@ -1732,24 +1686,22 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="43" t="inlineStr">
-        <is>
-          <t>04/07/2025</t>
-        </is>
-      </c>
-      <c r="B36" s="14" t="n">
+      <c r="A36" s="43" t="n">
+        <v>45754</v>
+      </c>
+      <c r="B36" s="56" t="n">
         <v>130752</v>
       </c>
-      <c r="C36" s="14" t="n">
+      <c r="C36" s="56" t="n">
         <v>15874</v>
       </c>
-      <c r="D36" s="14" t="n">
+      <c r="D36" s="56" t="n">
         <v>12681</v>
       </c>
-      <c r="E36" s="14" t="n">
+      <c r="E36" s="56" t="n">
         <v>18456</v>
       </c>
-      <c r="F36" s="14" t="n">
+      <c r="F36" s="56" t="n">
         <v>14505</v>
       </c>
       <c r="G36" s="14">
@@ -1762,24 +1714,22 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="43" t="inlineStr">
-        <is>
-          <t>04/14/2025</t>
-        </is>
-      </c>
-      <c r="B37" s="14" t="n">
+      <c r="A37" s="43" t="n">
+        <v>45761</v>
+      </c>
+      <c r="B37" s="56" t="n">
         <v>134703</v>
       </c>
-      <c r="C37" s="14" t="n">
+      <c r="C37" s="56" t="n">
         <v>14573</v>
       </c>
-      <c r="D37" s="14" t="n">
+      <c r="D37" s="56" t="n">
         <v>13129</v>
       </c>
-      <c r="E37" s="14" t="n">
+      <c r="E37" s="56" t="n">
         <v>17849</v>
       </c>
-      <c r="F37" s="14" t="n">
+      <c r="F37" s="56" t="n">
         <v>14594</v>
       </c>
       <c r="G37" s="14">
@@ -1792,24 +1742,22 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="43" t="inlineStr">
-        <is>
-          <t>04/21/2025</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="n">
+      <c r="A38" s="43" t="n">
+        <v>45768</v>
+      </c>
+      <c r="B38" s="56" t="n">
         <v>137958</v>
       </c>
-      <c r="C38" s="14" t="n">
+      <c r="C38" s="56" t="n">
         <v>14857</v>
       </c>
-      <c r="D38" s="14" t="n">
+      <c r="D38" s="56" t="n">
         <v>11916</v>
       </c>
-      <c r="E38" s="14" t="n">
+      <c r="E38" s="56" t="n">
         <v>17165</v>
       </c>
-      <c r="F38" s="14" t="n">
+      <c r="F38" s="56" t="n">
         <v>14136</v>
       </c>
       <c r="G38" s="14">
@@ -1822,24 +1770,22 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="43" t="inlineStr">
-        <is>
-          <t>04/28/2025</t>
-        </is>
-      </c>
-      <c r="B39" s="14" t="n">
+      <c r="A39" s="43" t="n">
+        <v>45775</v>
+      </c>
+      <c r="B39" s="56" t="n">
         <v>140987</v>
       </c>
-      <c r="C39" s="14" t="n">
+      <c r="C39" s="56" t="n">
         <v>13452</v>
       </c>
-      <c r="D39" s="14" t="n">
+      <c r="D39" s="56" t="n">
         <v>11244</v>
       </c>
-      <c r="E39" s="14" t="n">
+      <c r="E39" s="56" t="n">
         <v>16760</v>
       </c>
-      <c r="F39" s="14" t="n">
+      <c r="F39" s="56" t="n">
         <v>13400</v>
       </c>
       <c r="G39" s="14">
@@ -1852,24 +1798,22 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="43" t="inlineStr">
-        <is>
-          <t>05/05/2025</t>
-        </is>
-      </c>
-      <c r="B40" s="14" t="n">
+      <c r="A40" s="43" t="n">
+        <v>45782</v>
+      </c>
+      <c r="B40" s="56" t="n">
         <v>144347</v>
       </c>
-      <c r="C40" s="14" t="n">
+      <c r="C40" s="56" t="n">
         <v>14810</v>
       </c>
-      <c r="D40" s="14" t="n">
+      <c r="D40" s="56" t="n">
         <v>10593</v>
       </c>
-      <c r="E40" s="14" t="n">
+      <c r="E40" s="56" t="n">
         <v>17616</v>
       </c>
-      <c r="F40" s="14" t="n">
+      <c r="F40" s="56" t="n">
         <v>13861</v>
       </c>
       <c r="G40" s="14">
@@ -1882,24 +1826,22 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="43" t="inlineStr">
-        <is>
-          <t>05/12/2025</t>
-        </is>
-      </c>
-      <c r="B41" s="14" t="n">
+      <c r="A41" s="43" t="n">
+        <v>45789</v>
+      </c>
+      <c r="B41" s="56" t="n">
         <v>148102</v>
       </c>
-      <c r="C41" s="14" t="n">
+      <c r="C41" s="56" t="n">
         <v>14828</v>
       </c>
-      <c r="D41" s="14" t="n">
+      <c r="D41" s="56" t="n">
         <v>11551</v>
       </c>
-      <c r="E41" s="14" t="n">
+      <c r="E41" s="56" t="n">
         <v>16988</v>
       </c>
-      <c r="F41" s="14" t="n">
+      <c r="F41" s="56" t="n">
         <v>14487</v>
       </c>
       <c r="G41" s="14">
@@ -1912,24 +1854,22 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="43" t="inlineStr">
-        <is>
-          <t>05/19/2025</t>
-        </is>
-      </c>
-      <c r="B42" s="14" t="n">
+      <c r="A42" s="43" t="n">
+        <v>45796</v>
+      </c>
+      <c r="B42" s="56" t="n">
         <v>150603</v>
       </c>
-      <c r="C42" s="14" t="n">
+      <c r="C42" s="56" t="n">
         <v>13995</v>
       </c>
-      <c r="D42" s="14" t="n">
+      <c r="D42" s="56" t="n">
         <v>11028</v>
       </c>
-      <c r="E42" s="14" t="n">
+      <c r="E42" s="56" t="n">
         <v>17848</v>
       </c>
-      <c r="F42" s="14" t="n">
+      <c r="F42" s="56" t="n">
         <v>14395</v>
       </c>
       <c r="G42" s="14">
@@ -1942,24 +1882,22 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="43" t="inlineStr">
-        <is>
-          <t>05/26/2025</t>
-        </is>
-      </c>
-      <c r="B43" s="14" t="n">
+      <c r="A43" s="43" t="n">
+        <v>45803</v>
+      </c>
+      <c r="B43" s="56" t="n">
         <v>154056</v>
       </c>
-      <c r="C43" s="14" t="n">
+      <c r="C43" s="56" t="n">
         <v>15854</v>
       </c>
-      <c r="D43" s="14" t="n">
+      <c r="D43" s="56" t="n">
         <v>11534</v>
       </c>
-      <c r="E43" s="14" t="n">
+      <c r="E43" s="56" t="n">
         <v>19020</v>
       </c>
-      <c r="F43" s="14" t="n">
+      <c r="F43" s="56" t="n">
         <v>14476</v>
       </c>
       <c r="G43" s="14">
@@ -1972,24 +1910,22 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="43" t="inlineStr">
-        <is>
-          <t>06/02/2025</t>
-        </is>
-      </c>
-      <c r="B44" s="14" t="n">
+      <c r="A44" s="43" t="n">
+        <v>45810</v>
+      </c>
+      <c r="B44" s="56" t="n">
         <v>158600</v>
       </c>
-      <c r="C44" s="14" t="n">
+      <c r="C44" s="56" t="n">
         <v>15894</v>
       </c>
-      <c r="D44" s="14" t="n">
+      <c r="D44" s="56" t="n">
         <v>10230</v>
       </c>
-      <c r="E44" s="14" t="n">
+      <c r="E44" s="56" t="n">
         <v>18256</v>
       </c>
-      <c r="F44" s="14" t="n">
+      <c r="F44" s="56" t="n">
         <v>13816</v>
       </c>
       <c r="G44" s="14">
@@ -2002,24 +1938,22 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="43" t="inlineStr">
-        <is>
-          <t>06/09/2025</t>
-        </is>
-      </c>
-      <c r="B45" s="14" t="n">
+      <c r="A45" s="43" t="n">
+        <v>45817</v>
+      </c>
+      <c r="B45" s="56" t="n">
         <v>163040</v>
       </c>
-      <c r="C45" s="14" t="n">
+      <c r="C45" s="56" t="n">
         <v>15706</v>
       </c>
-      <c r="D45" s="14" t="n">
+      <c r="D45" s="56" t="n">
         <v>12238</v>
       </c>
-      <c r="E45" s="14" t="n">
+      <c r="E45" s="56" t="n">
         <v>17987</v>
       </c>
-      <c r="F45" s="14" t="n">
+      <c r="F45" s="56" t="n">
         <v>13939</v>
       </c>
       <c r="G45" s="14">
@@ -2032,24 +1966,22 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="43" t="inlineStr">
-        <is>
-          <t>06/16/2025</t>
-        </is>
-      </c>
-      <c r="B46" s="14" t="n">
+      <c r="A46" s="43" t="n">
+        <v>45824</v>
+      </c>
+      <c r="B46" s="56" t="n">
         <v>167088</v>
       </c>
-      <c r="C46" s="14" t="n">
+      <c r="C46" s="56" t="n">
         <v>14323</v>
       </c>
-      <c r="D46" s="14" t="n">
+      <c r="D46" s="56" t="n">
         <v>10924</v>
       </c>
-      <c r="E46" s="14" t="n">
+      <c r="E46" s="56" t="n">
         <v>18476</v>
       </c>
-      <c r="F46" s="14" t="n">
+      <c r="F46" s="56" t="n">
         <v>14138</v>
       </c>
       <c r="G46" s="14">
@@ -2062,24 +1994,22 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="43" t="inlineStr">
-        <is>
-          <t>06/23/2025</t>
-        </is>
-      </c>
-      <c r="B47" s="14" t="n">
+      <c r="A47" s="43" t="n">
+        <v>45831</v>
+      </c>
+      <c r="B47" s="56" t="n">
         <v>171426</v>
       </c>
-      <c r="C47" s="14" t="n">
+      <c r="C47" s="56" t="n">
         <v>15852</v>
       </c>
-      <c r="D47" s="14" t="n">
+      <c r="D47" s="56" t="n">
         <v>11233</v>
       </c>
-      <c r="E47" s="14" t="n">
+      <c r="E47" s="56" t="n">
         <v>17619</v>
       </c>
-      <c r="F47" s="14" t="n">
+      <c r="F47" s="56" t="n">
         <v>13696</v>
       </c>
       <c r="G47" s="14">
@@ -2092,24 +2022,22 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="43" t="inlineStr">
-        <is>
-          <t>06/30/2025</t>
-        </is>
-      </c>
-      <c r="B48" s="14" t="n">
+      <c r="A48" s="43" t="n">
+        <v>45838</v>
+      </c>
+      <c r="B48" s="56" t="n">
         <v>175349</v>
       </c>
-      <c r="C48" s="14" t="n">
+      <c r="C48" s="56" t="n">
         <v>13553</v>
       </c>
-      <c r="D48" s="14" t="n">
+      <c r="D48" s="56" t="n">
         <v>12751</v>
       </c>
-      <c r="E48" s="14" t="n">
+      <c r="E48" s="56" t="n">
         <v>17137</v>
       </c>
-      <c r="F48" s="14" t="n">
+      <c r="F48" s="56" t="n">
         <v>15003</v>
       </c>
       <c r="G48" s="14">
@@ -2122,24 +2050,22 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="43" t="inlineStr">
-        <is>
-          <t>07/07/2025</t>
-        </is>
-      </c>
-      <c r="B49" s="14" t="n">
+      <c r="A49" s="43" t="n">
+        <v>45845</v>
+      </c>
+      <c r="B49" s="56" t="n">
         <v>177483</v>
       </c>
-      <c r="C49" s="14" t="n">
+      <c r="C49" s="56" t="n">
         <v>15488</v>
       </c>
-      <c r="D49" s="14" t="n">
+      <c r="D49" s="56" t="n">
         <v>12193</v>
       </c>
-      <c r="E49" s="14" t="n">
+      <c r="E49" s="56" t="n">
         <v>17692</v>
       </c>
-      <c r="F49" s="14" t="n">
+      <c r="F49" s="56" t="n">
         <v>14725</v>
       </c>
       <c r="G49" s="14">
@@ -2152,24 +2078,22 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="43" t="inlineStr">
-        <is>
-          <t>07/14/2025</t>
-        </is>
-      </c>
-      <c r="B50" s="14" t="n">
+      <c r="A50" s="43" t="n">
+        <v>45852</v>
+      </c>
+      <c r="B50" s="56" t="n">
         <v>180450</v>
       </c>
-      <c r="C50" s="14" t="n">
+      <c r="C50" s="56" t="n">
         <v>15022</v>
       </c>
-      <c r="D50" s="14" t="n">
+      <c r="D50" s="56" t="n">
         <v>11956</v>
       </c>
-      <c r="E50" s="14" t="n">
+      <c r="E50" s="56" t="n">
         <v>18559</v>
       </c>
-      <c r="F50" s="14" t="n">
+      <c r="F50" s="56" t="n">
         <v>14153</v>
       </c>
       <c r="G50" s="14">
@@ -2182,24 +2106,22 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="43" t="inlineStr">
-        <is>
-          <t>07/21/2025</t>
-        </is>
-      </c>
-      <c r="B51" s="14" t="n">
+      <c r="A51" s="43" t="n">
+        <v>45859</v>
+      </c>
+      <c r="B51" s="56" t="n">
         <v>184856</v>
       </c>
-      <c r="C51" s="14" t="n">
+      <c r="C51" s="56" t="n">
         <v>14269</v>
       </c>
-      <c r="D51" s="14" t="n">
+      <c r="D51" s="56" t="n">
         <v>11177</v>
       </c>
-      <c r="E51" s="14" t="n">
+      <c r="E51" s="56" t="n">
         <v>16200</v>
       </c>
-      <c r="F51" s="14" t="n">
+      <c r="F51" s="56" t="n">
         <v>14930</v>
       </c>
       <c r="G51" s="14">
@@ -2212,24 +2134,22 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="43" t="inlineStr">
-        <is>
-          <t>07/28/2025</t>
-        </is>
-      </c>
-      <c r="B52" s="14" t="n">
+      <c r="A52" s="43" t="n">
+        <v>45866</v>
+      </c>
+      <c r="B52" s="56" t="n">
         <v>186126</v>
       </c>
-      <c r="C52" s="14" t="n">
+      <c r="C52" s="56" t="n">
         <v>13988</v>
       </c>
-      <c r="D52" s="14" t="n">
+      <c r="D52" s="56" t="n">
         <v>13046</v>
       </c>
-      <c r="E52" s="14" t="n">
+      <c r="E52" s="56" t="n">
         <v>16263</v>
       </c>
-      <c r="F52" s="14" t="n">
+      <c r="F52" s="56" t="n">
         <v>14616</v>
       </c>
       <c r="G52" s="14">
@@ -2242,24 +2162,22 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="43" t="inlineStr">
-        <is>
-          <t>08/04/2025</t>
-        </is>
-      </c>
-      <c r="B53" s="14" t="n">
+      <c r="A53" s="43" t="n">
+        <v>45873</v>
+      </c>
+      <c r="B53" s="56" t="n">
         <v>187773</v>
       </c>
-      <c r="C53" s="14" t="n">
+      <c r="C53" s="56" t="n">
         <v>13890</v>
       </c>
-      <c r="D53" s="14" t="n">
+      <c r="D53" s="56" t="n">
         <v>12900</v>
       </c>
-      <c r="E53" s="14" t="n">
+      <c r="E53" s="56" t="n">
         <v>18024</v>
       </c>
-      <c r="F53" s="14" t="n">
+      <c r="F53" s="56" t="n">
         <v>14885</v>
       </c>
       <c r="G53" s="14">
@@ -2272,24 +2190,22 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="43" t="inlineStr">
-        <is>
-          <t>08/11/2025</t>
-        </is>
-      </c>
-      <c r="B54" s="14" t="n">
+      <c r="A54" s="43" t="n">
+        <v>45880</v>
+      </c>
+      <c r="B54" s="56" t="n">
         <v>190912</v>
       </c>
-      <c r="C54" s="14" t="n">
+      <c r="C54" s="56" t="n">
         <v>16110</v>
       </c>
-      <c r="D54" s="14" t="n">
+      <c r="D54" s="56" t="n">
         <v>12023</v>
       </c>
-      <c r="E54" s="14" t="n">
+      <c r="E54" s="56" t="n">
         <v>17922</v>
       </c>
-      <c r="F54" s="14" t="n">
+      <c r="F54" s="56" t="n">
         <v>13767</v>
       </c>
       <c r="G54" s="14">
@@ -2302,24 +2218,22 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="43" t="inlineStr">
-        <is>
-          <t>08/18/2025</t>
-        </is>
-      </c>
-      <c r="B55" s="14" t="n">
+      <c r="A55" s="43" t="n">
+        <v>45887</v>
+      </c>
+      <c r="B55" s="56" t="n">
         <v>195067</v>
       </c>
-      <c r="C55" s="14" t="n">
+      <c r="C55" s="56" t="n">
         <v>14046</v>
       </c>
-      <c r="D55" s="14" t="n">
+      <c r="D55" s="56" t="n">
         <v>12378</v>
       </c>
-      <c r="E55" s="14" t="n">
+      <c r="E55" s="56" t="n">
         <v>17464</v>
       </c>
-      <c r="F55" s="14" t="n">
+      <c r="F55" s="56" t="n">
         <v>14833</v>
       </c>
       <c r="G55" s="14">
@@ -2332,24 +2246,22 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="43" t="inlineStr">
-        <is>
-          <t>08/25/2025</t>
-        </is>
-      </c>
-      <c r="B56" s="14" t="n">
+      <c r="A56" s="43" t="n">
+        <v>45894</v>
+      </c>
+      <c r="B56" s="56" t="n">
         <v>197698</v>
       </c>
-      <c r="C56" s="14" t="n">
+      <c r="C56" s="56" t="n">
         <v>15073</v>
       </c>
-      <c r="D56" s="14" t="n">
+      <c r="D56" s="56" t="n">
         <v>11870</v>
       </c>
-      <c r="E56" s="14" t="n">
+      <c r="E56" s="56" t="n">
         <v>17834</v>
       </c>
-      <c r="F56" s="14" t="n">
+      <c r="F56" s="56" t="n">
         <v>14814</v>
       </c>
       <c r="G56" s="14">
@@ -2362,24 +2274,22 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="43" t="inlineStr">
-        <is>
-          <t>09/01/2025</t>
-        </is>
-      </c>
-      <c r="B57" s="14" t="n">
+      <c r="A57" s="43" t="n">
+        <v>45901</v>
+      </c>
+      <c r="B57" s="56" t="n">
         <v>200718</v>
       </c>
-      <c r="C57" s="14" t="n">
+      <c r="C57" s="56" t="n">
         <v>15661</v>
       </c>
-      <c r="D57" s="14" t="n">
+      <c r="D57" s="56" t="n">
         <v>11471</v>
       </c>
-      <c r="E57" s="14" t="n">
+      <c r="E57" s="56" t="n">
         <v>18954</v>
       </c>
-      <c r="F57" s="14" t="n">
+      <c r="F57" s="56" t="n">
         <v>13901</v>
       </c>
       <c r="G57" s="14">
@@ -2392,24 +2302,22 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="43" t="inlineStr">
-        <is>
-          <t>09/08/2025</t>
-        </is>
-      </c>
-      <c r="B58" s="14" t="n">
+      <c r="A58" s="43" t="n">
+        <v>45908</v>
+      </c>
+      <c r="B58" s="56" t="n">
         <v>205771</v>
       </c>
-      <c r="C58" s="14" t="n">
+      <c r="C58" s="56" t="n">
         <v>14722</v>
       </c>
-      <c r="D58" s="14" t="n">
+      <c r="D58" s="56" t="n">
         <v>13517</v>
       </c>
-      <c r="E58" s="14" t="n">
+      <c r="E58" s="56" t="n">
         <v>17430</v>
       </c>
-      <c r="F58" s="14" t="n">
+      <c r="F58" s="56" t="n">
         <v>15325</v>
       </c>
       <c r="G58" s="14">
@@ -2422,24 +2330,22 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="43" t="inlineStr">
-        <is>
-          <t>09/15/2025</t>
-        </is>
-      </c>
-      <c r="B59" s="14" t="n">
+      <c r="A59" s="43" t="n">
+        <v>45915</v>
+      </c>
+      <c r="B59" s="56" t="n">
         <v>207876</v>
       </c>
-      <c r="C59" s="14" t="n">
+      <c r="C59" s="56" t="n">
         <v>14659</v>
       </c>
-      <c r="D59" s="14" t="n">
+      <c r="D59" s="56" t="n">
         <v>11181</v>
       </c>
-      <c r="E59" s="14" t="n">
+      <c r="E59" s="56" t="n">
         <v>18252</v>
       </c>
-      <c r="F59" s="14" t="n">
+      <c r="F59" s="56" t="n">
         <v>14978</v>
       </c>
       <c r="G59" s="14">
@@ -2452,24 +2358,22 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="43" t="inlineStr">
-        <is>
-          <t>09/22/2025</t>
-        </is>
-      </c>
-      <c r="B60" s="14" t="n">
+      <c r="A60" s="43" t="n">
+        <v>45922</v>
+      </c>
+      <c r="B60" s="56" t="n">
         <v>211150</v>
       </c>
-      <c r="C60" s="14" t="n">
+      <c r="C60" s="56" t="n">
         <v>14652</v>
       </c>
-      <c r="D60" s="14" t="n">
+      <c r="D60" s="56" t="n">
         <v>12753</v>
       </c>
-      <c r="E60" s="14" t="n">
+      <c r="E60" s="56" t="n">
         <v>18707</v>
       </c>
-      <c r="F60" s="14" t="n">
+      <c r="F60" s="56" t="n">
         <v>14054</v>
       </c>
       <c r="G60" s="14">
@@ -2482,24 +2386,22 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="43" t="inlineStr">
-        <is>
-          <t>09/29/2025</t>
-        </is>
-      </c>
-      <c r="B61" s="14" t="n">
+      <c r="A61" s="43" t="n">
+        <v>45929</v>
+      </c>
+      <c r="B61" s="56" t="n">
         <v>215803</v>
       </c>
-      <c r="C61" s="14" t="n">
+      <c r="C61" s="56" t="n">
         <v>14794</v>
       </c>
-      <c r="D61" s="14" t="n">
+      <c r="D61" s="56" t="n">
         <v>12038</v>
       </c>
-      <c r="E61" s="14" t="n">
+      <c r="E61" s="56" t="n">
         <v>17813</v>
       </c>
-      <c r="F61" s="14" t="n">
+      <c r="F61" s="56" t="n">
         <v>15250</v>
       </c>
       <c r="G61" s="14">
@@ -2512,24 +2414,22 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="43" t="inlineStr">
-        <is>
-          <t>10/06/2025</t>
-        </is>
-      </c>
-      <c r="B62" s="14" t="n">
+      <c r="A62" s="43" t="n">
+        <v>45936</v>
+      </c>
+      <c r="B62" s="56" t="n">
         <v>218366</v>
       </c>
-      <c r="C62" s="14" t="n">
+      <c r="C62" s="56" t="n">
         <v>15475</v>
       </c>
-      <c r="D62" s="14" t="n">
+      <c r="D62" s="56" t="n">
         <v>13487</v>
       </c>
-      <c r="E62" s="14" t="n">
+      <c r="E62" s="56" t="n">
         <v>18183</v>
       </c>
-      <c r="F62" s="14" t="n">
+      <c r="F62" s="56" t="n">
         <v>15166</v>
       </c>
       <c r="G62" s="14">
@@ -2542,24 +2442,22 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="43" t="inlineStr">
-        <is>
-          <t>10/13/2025</t>
-        </is>
-      </c>
-      <c r="B63" s="14" t="n">
+      <c r="A63" s="43" t="n">
+        <v>45943</v>
+      </c>
+      <c r="B63" s="56" t="n">
         <v>221383</v>
       </c>
-      <c r="C63" s="14" t="n">
+      <c r="C63" s="56" t="n">
         <v>14013</v>
       </c>
-      <c r="D63" s="14" t="n">
+      <c r="D63" s="56" t="n">
         <v>12831</v>
       </c>
-      <c r="E63" s="14" t="n">
+      <c r="E63" s="56" t="n">
         <v>18169</v>
       </c>
-      <c r="F63" s="14" t="n">
+      <c r="F63" s="56" t="n">
         <v>14661</v>
       </c>
       <c r="G63" s="14">
@@ -2572,24 +2470,22 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="43" t="inlineStr">
-        <is>
-          <t>10/20/2025</t>
-        </is>
-      </c>
-      <c r="B64" s="14" t="n">
+      <c r="A64" s="43" t="n">
+        <v>45950</v>
+      </c>
+      <c r="B64" s="56" t="n">
         <v>224891</v>
       </c>
-      <c r="C64" s="14" t="n">
+      <c r="C64" s="56" t="n">
         <v>15133</v>
       </c>
-      <c r="D64" s="14" t="n">
+      <c r="D64" s="56" t="n">
         <v>11127</v>
       </c>
-      <c r="E64" s="14" t="n">
+      <c r="E64" s="56" t="n">
         <v>17393</v>
       </c>
-      <c r="F64" s="14" t="n">
+      <c r="F64" s="56" t="n">
         <v>14240</v>
       </c>
       <c r="G64" s="14">
@@ -2602,24 +2498,22 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="43" t="inlineStr">
-        <is>
-          <t>10/27/2025</t>
-        </is>
-      </c>
-      <c r="B65" s="14" t="n">
+      <c r="A65" s="43" t="n">
+        <v>45957</v>
+      </c>
+      <c r="B65" s="56" t="n">
         <v>228044</v>
       </c>
-      <c r="C65" s="14" t="n">
+      <c r="C65" s="56" t="n">
         <v>16830</v>
       </c>
-      <c r="D65" s="14" t="n">
+      <c r="D65" s="56" t="n">
         <v>12830</v>
       </c>
-      <c r="E65" s="14" t="n">
+      <c r="E65" s="56" t="n">
         <v>18774</v>
       </c>
-      <c r="F65" s="14" t="n">
+      <c r="F65" s="56" t="n">
         <v>15407</v>
       </c>
       <c r="G65" s="14">
@@ -2632,24 +2526,22 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="43" t="inlineStr">
-        <is>
-          <t>11/03/2025</t>
-        </is>
-      </c>
-      <c r="B66" s="14" t="n">
+      <c r="A66" s="43" t="n">
+        <v>45964</v>
+      </c>
+      <c r="B66" s="56" t="n">
         <v>231411</v>
       </c>
-      <c r="C66" s="14" t="n">
+      <c r="C66" s="56" t="n">
         <v>13782</v>
       </c>
-      <c r="D66" s="14" t="n">
+      <c r="D66" s="56" t="n">
         <v>10805</v>
       </c>
-      <c r="E66" s="14" t="n">
+      <c r="E66" s="56" t="n">
         <v>17498</v>
       </c>
-      <c r="F66" s="14" t="n">
+      <c r="F66" s="56" t="n">
         <v>14167</v>
       </c>
       <c r="G66" s="14">
@@ -2662,24 +2554,22 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="43" t="inlineStr">
-        <is>
-          <t>11/10/2025</t>
-        </is>
-      </c>
-      <c r="B67" s="14" t="n">
+      <c r="A67" s="43" t="n">
+        <v>45971</v>
+      </c>
+      <c r="B67" s="56" t="n">
         <v>234742</v>
       </c>
-      <c r="C67" s="14" t="n">
+      <c r="C67" s="56" t="n">
         <v>15500</v>
       </c>
-      <c r="D67" s="14" t="n">
+      <c r="D67" s="56" t="n">
         <v>12307</v>
       </c>
-      <c r="E67" s="14" t="n">
+      <c r="E67" s="56" t="n">
         <v>17384</v>
       </c>
-      <c r="F67" s="14" t="n">
+      <c r="F67" s="56" t="n">
         <v>14700</v>
       </c>
       <c r="G67" s="14">
@@ -2692,24 +2582,22 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="43" t="inlineStr">
-        <is>
-          <t>11/17/2025</t>
-        </is>
-      </c>
-      <c r="B68" s="14" t="n">
+      <c r="A68" s="43" t="n">
+        <v>45978</v>
+      </c>
+      <c r="B68" s="56" t="n">
         <v>237426</v>
       </c>
-      <c r="C68" s="14" t="n">
+      <c r="C68" s="56" t="n">
         <v>16905</v>
       </c>
-      <c r="D68" s="14" t="n">
+      <c r="D68" s="56" t="n">
         <v>13861</v>
       </c>
-      <c r="E68" s="14" t="n">
+      <c r="E68" s="56" t="n">
         <v>18794</v>
       </c>
-      <c r="F68" s="14" t="n">
+      <c r="F68" s="56" t="n">
         <v>15817</v>
       </c>
       <c r="G68" s="14">
@@ -2722,24 +2610,22 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="43" t="inlineStr">
-        <is>
-          <t>11/24/2025</t>
-        </is>
-      </c>
-      <c r="B69" s="14" t="n">
+      <c r="A69" s="43" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B69" s="56" t="n">
         <v>240403</v>
       </c>
-      <c r="C69" s="14" t="n">
+      <c r="C69" s="56" t="n">
         <v>17465</v>
       </c>
-      <c r="D69" s="14" t="n">
+      <c r="D69" s="56" t="n">
         <v>13521</v>
       </c>
-      <c r="E69" s="14" t="n">
+      <c r="E69" s="56" t="n">
         <v>19687</v>
       </c>
-      <c r="F69" s="14" t="n">
+      <c r="F69" s="56" t="n">
         <v>15430</v>
       </c>
       <c r="G69" s="14">
@@ -2752,24 +2638,22 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="43" t="inlineStr">
-        <is>
-          <t>12/01/2025</t>
-        </is>
-      </c>
-      <c r="B70" s="14" t="n">
+      <c r="A70" s="43" t="n">
+        <v>45992</v>
+      </c>
+      <c r="B70" s="56" t="n">
         <v>244660</v>
       </c>
-      <c r="C70" s="14" t="n">
+      <c r="C70" s="56" t="n">
         <v>15352</v>
       </c>
-      <c r="D70" s="14" t="n">
+      <c r="D70" s="56" t="n">
         <v>11740</v>
       </c>
-      <c r="E70" s="14" t="n">
+      <c r="E70" s="56" t="n">
         <v>18910</v>
       </c>
-      <c r="F70" s="14" t="n">
+      <c r="F70" s="56" t="n">
         <v>15652</v>
       </c>
       <c r="G70" s="14">
@@ -2782,24 +2666,22 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="43" t="inlineStr">
-        <is>
-          <t>12/08/2025</t>
-        </is>
-      </c>
-      <c r="B71" s="14" t="n">
+      <c r="A71" s="43" t="n">
+        <v>45999</v>
+      </c>
+      <c r="B71" s="56" t="n">
         <v>247918</v>
       </c>
-      <c r="C71" s="14" t="n">
+      <c r="C71" s="56" t="n">
         <v>16920</v>
       </c>
-      <c r="D71" s="14" t="n">
+      <c r="D71" s="56" t="n">
         <v>14373</v>
       </c>
-      <c r="E71" s="14" t="n">
+      <c r="E71" s="56" t="n">
         <v>20105</v>
       </c>
-      <c r="F71" s="14" t="n">
+      <c r="F71" s="56" t="n">
         <v>16070</v>
       </c>
       <c r="G71" s="14">
@@ -2812,24 +2694,22 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="43" t="inlineStr">
-        <is>
-          <t>12/15/2025</t>
-        </is>
-      </c>
-      <c r="B72" s="14" t="n">
+      <c r="A72" s="43" t="n">
+        <v>46006</v>
+      </c>
+      <c r="B72" s="56" t="n">
         <v>251953</v>
       </c>
-      <c r="C72" s="14" t="n">
+      <c r="C72" s="56" t="n">
         <v>15424</v>
       </c>
-      <c r="D72" s="14" t="n">
+      <c r="D72" s="56" t="n">
         <v>11991</v>
       </c>
-      <c r="E72" s="14" t="n">
+      <c r="E72" s="56" t="n">
         <v>19349</v>
       </c>
-      <c r="F72" s="14" t="n">
+      <c r="F72" s="56" t="n">
         <v>14643</v>
       </c>
       <c r="G72" s="14">
@@ -2842,24 +2722,22 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="43" t="inlineStr">
-        <is>
-          <t>12/22/2025</t>
-        </is>
-      </c>
-      <c r="B73" s="14" t="n">
+      <c r="A73" s="43" t="n">
+        <v>46013</v>
+      </c>
+      <c r="B73" s="56" t="n">
         <v>256659</v>
       </c>
-      <c r="C73" s="14" t="n">
+      <c r="C73" s="56" t="n">
         <v>14165</v>
       </c>
-      <c r="D73" s="14" t="n">
+      <c r="D73" s="56" t="n">
         <v>13442</v>
       </c>
-      <c r="E73" s="14" t="n">
+      <c r="E73" s="56" t="n">
         <v>18388</v>
       </c>
-      <c r="F73" s="14" t="n">
+      <c r="F73" s="56" t="n">
         <v>15382</v>
       </c>
       <c r="G73" s="14">
@@ -2872,24 +2750,22 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="43" t="inlineStr">
-        <is>
-          <t>12/29/2025</t>
-        </is>
-      </c>
-      <c r="B74" s="14" t="n">
+      <c r="A74" s="43" t="n">
+        <v>46020</v>
+      </c>
+      <c r="B74" s="56" t="n">
         <v>259665</v>
       </c>
-      <c r="C74" s="14" t="n">
+      <c r="C74" s="56" t="n">
         <v>15540</v>
       </c>
-      <c r="D74" s="14" t="n">
+      <c r="D74" s="56" t="n">
         <v>12266</v>
       </c>
-      <c r="E74" s="14" t="n">
+      <c r="E74" s="56" t="n">
         <v>19865</v>
       </c>
-      <c r="F74" s="14" t="n">
+      <c r="F74" s="56" t="n">
         <v>15811</v>
       </c>
       <c r="G74" s="14">
@@ -2902,24 +2778,22 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="43" t="inlineStr">
-        <is>
-          <t>01/05/2026</t>
-        </is>
-      </c>
-      <c r="B75" s="14" t="n">
+      <c r="A75" s="43" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B75" s="56" t="n">
         <v>263719</v>
       </c>
-      <c r="C75" s="14" t="n">
+      <c r="C75" s="56" t="n">
         <v>15662</v>
       </c>
-      <c r="D75" s="14" t="n">
+      <c r="D75" s="56" t="n">
         <v>13921</v>
       </c>
-      <c r="E75" s="14" t="n">
+      <c r="E75" s="56" t="n">
         <v>19507</v>
       </c>
-      <c r="F75" s="14" t="n">
+      <c r="F75" s="56" t="n">
         <v>16187</v>
       </c>
       <c r="G75" s="14">
@@ -2932,24 +2806,22 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="43" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
-        </is>
-      </c>
-      <c r="B76" s="14" t="n">
+      <c r="A76" s="43" t="n">
+        <v>46034</v>
+      </c>
+      <c r="B76" s="56" t="n">
         <v>267039</v>
       </c>
-      <c r="C76" s="14" t="n">
+      <c r="C76" s="56" t="n">
         <v>14562</v>
       </c>
-      <c r="D76" s="14" t="n">
+      <c r="D76" s="56" t="n">
         <v>14803</v>
       </c>
-      <c r="E76" s="14" t="n">
+      <c r="E76" s="56" t="n">
         <v>18853</v>
       </c>
-      <c r="F76" s="14" t="n">
+      <c r="F76" s="56" t="n">
         <v>16302</v>
       </c>
       <c r="G76" s="14">
@@ -2962,24 +2834,22 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="43" t="inlineStr">
-        <is>
-          <t>01/19/2026</t>
-        </is>
-      </c>
-      <c r="B77" s="14" t="n">
+      <c r="A77" s="43" t="n">
+        <v>46041</v>
+      </c>
+      <c r="B77" s="56" t="n">
         <v>269590</v>
       </c>
-      <c r="C77" s="14" t="n">
+      <c r="C77" s="56" t="n">
         <v>14993</v>
       </c>
-      <c r="D77" s="14" t="n">
+      <c r="D77" s="56" t="n">
         <v>13911</v>
       </c>
-      <c r="E77" s="14" t="n">
+      <c r="E77" s="56" t="n">
         <v>17993</v>
       </c>
-      <c r="F77" s="14" t="n">
+      <c r="F77" s="56" t="n">
         <v>16677</v>
       </c>
       <c r="G77" s="14">
@@ -2992,24 +2862,22 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="43" t="inlineStr">
-        <is>
-          <t>01/26/2026</t>
-        </is>
-      </c>
-      <c r="B78" s="14" t="n">
+      <c r="A78" s="43" t="n">
+        <v>46048</v>
+      </c>
+      <c r="B78" s="56" t="n">
         <v>270906</v>
       </c>
-      <c r="C78" s="14" t="n">
+      <c r="C78" s="56" t="n">
         <v>15605</v>
       </c>
-      <c r="D78" s="14" t="n">
+      <c r="D78" s="56" t="n">
         <v>13902</v>
       </c>
-      <c r="E78" s="14" t="n">
+      <c r="E78" s="56" t="n">
         <v>17714</v>
       </c>
-      <c r="F78" s="14" t="n">
+      <c r="F78" s="56" t="n">
         <v>15722</v>
       </c>
       <c r="G78" s="14">
@@ -3022,24 +2890,22 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="43" t="inlineStr">
-        <is>
-          <t>02/02/2026</t>
-        </is>
-      </c>
-      <c r="B79" s="14" t="n">
+      <c r="A79" s="43" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B79" s="56" t="n">
         <v>272898</v>
       </c>
-      <c r="C79" s="14" t="n">
+      <c r="C79" s="56" t="n">
         <v>14253</v>
       </c>
-      <c r="D79" s="14" t="n">
+      <c r="D79" s="56" t="n">
         <v>13649</v>
       </c>
-      <c r="E79" s="14" t="n">
+      <c r="E79" s="56" t="n">
         <v>18508</v>
       </c>
-      <c r="F79" s="14" t="n">
+      <c r="F79" s="56" t="n">
         <v>16670</v>
       </c>
       <c r="G79" s="14">
@@ -3052,24 +2918,22 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="43" t="inlineStr">
-        <is>
-          <t>02/09/2026</t>
-        </is>
-      </c>
-      <c r="B80" s="14" t="n">
+      <c r="A80" s="43" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B80" s="56" t="n">
         <v>274736</v>
       </c>
-      <c r="C80" s="14" t="n">
+      <c r="C80" s="56" t="n">
         <v>15317</v>
       </c>
-      <c r="D80" s="14" t="n">
+      <c r="D80" s="56" t="n">
         <v>14335</v>
       </c>
-      <c r="E80" s="14" t="n">
+      <c r="E80" s="56" t="n">
         <v>18997</v>
       </c>
-      <c r="F80" s="14" t="n">
+      <c r="F80" s="56" t="n">
         <v>15987</v>
       </c>
       <c r="G80" s="14">
@@ -3082,24 +2946,22 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="43" t="inlineStr">
-        <is>
-          <t>02/16/2026</t>
-        </is>
-      </c>
-      <c r="B81" s="14" t="n">
+      <c r="A81" s="43" t="n">
+        <v>46069</v>
+      </c>
+      <c r="B81" s="56" t="n">
         <v>277746</v>
       </c>
-      <c r="C81" s="14" t="n">
+      <c r="C81" s="56" t="n">
         <v>16251</v>
       </c>
-      <c r="D81" s="14" t="n">
+      <c r="D81" s="56" t="n">
         <v>12736</v>
       </c>
-      <c r="E81" s="14" t="n">
+      <c r="E81" s="56" t="n">
         <v>19001</v>
       </c>
-      <c r="F81" s="14" t="n">
+      <c r="F81" s="56" t="n">
         <v>15905</v>
       </c>
       <c r="G81" s="14">
@@ -3112,24 +2974,22 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="43" t="inlineStr">
-        <is>
-          <t>02/23/2026</t>
-        </is>
-      </c>
-      <c r="B82" s="14" t="n">
+      <c r="A82" s="43" t="n">
+        <v>46076</v>
+      </c>
+      <c r="B82" s="56" t="n">
         <v>280842</v>
       </c>
-      <c r="C82" s="14" t="n">
+      <c r="C82" s="56" t="n">
         <v>17754</v>
       </c>
-      <c r="D82" s="14" t="n">
+      <c r="D82" s="56" t="n">
         <v>13587</v>
       </c>
-      <c r="E82" s="14" t="n">
+      <c r="E82" s="56" t="n">
         <v>20679</v>
       </c>
-      <c r="F82" s="14" t="n">
+      <c r="F82" s="56" t="n">
         <v>15613</v>
       </c>
       <c r="G82" s="14">
@@ -3142,24 +3002,22 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="43" t="inlineStr">
-        <is>
-          <t>03/02/2026</t>
-        </is>
-      </c>
-      <c r="B83" s="14" t="n">
+      <c r="A83" s="43" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B83" s="56" t="n">
         <v>285908</v>
       </c>
-      <c r="C83" s="14" t="n">
+      <c r="C83" s="56" t="n">
         <v>16503</v>
       </c>
-      <c r="D83" s="14" t="n">
+      <c r="D83" s="56" t="n">
         <v>14799</v>
       </c>
-      <c r="E83" s="14" t="n">
+      <c r="E83" s="56" t="n">
         <v>19158</v>
       </c>
-      <c r="F83" s="14" t="n">
+      <c r="F83" s="56" t="n">
         <v>16738</v>
       </c>
       <c r="G83" s="14">
@@ -3172,24 +3030,22 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="43" t="inlineStr">
-        <is>
-          <t>03/09/2026</t>
-        </is>
-      </c>
-      <c r="B84" s="14" t="n">
+      <c r="A84" s="43" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B84" s="56" t="n">
         <v>288328</v>
       </c>
-      <c r="C84" s="14" t="n">
+      <c r="C84" s="56" t="n">
         <v>17555</v>
       </c>
-      <c r="D84" s="14" t="n">
+      <c r="D84" s="56" t="n">
         <v>11850</v>
       </c>
-      <c r="E84" s="14" t="n">
+      <c r="E84" s="56" t="n">
         <v>20705</v>
       </c>
-      <c r="F84" s="14" t="n">
+      <c r="F84" s="56" t="n">
         <v>15984</v>
       </c>
       <c r="G84" s="14">
@@ -3202,24 +3058,22 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="43" t="inlineStr">
-        <is>
-          <t>03/16/2026</t>
-        </is>
-      </c>
-      <c r="B85" s="14" t="n">
+      <c r="A85" s="43" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B85" s="56" t="n">
         <v>293049</v>
       </c>
-      <c r="C85" s="14" t="n">
+      <c r="C85" s="56" t="n">
         <v>16850</v>
       </c>
-      <c r="D85" s="14" t="n">
+      <c r="D85" s="56" t="n">
         <v>14493</v>
       </c>
-      <c r="E85" s="14" t="n">
+      <c r="E85" s="56" t="n">
         <v>20200</v>
       </c>
-      <c r="F85" s="14" t="n">
+      <c r="F85" s="56" t="n">
         <v>17221</v>
       </c>
       <c r="G85" s="14">
@@ -3232,24 +3086,22 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="43" t="inlineStr">
-        <is>
-          <t>03/23/2026</t>
-        </is>
-      </c>
-      <c r="B86" s="14" t="n">
+      <c r="A86" s="43" t="n">
+        <v>46104</v>
+      </c>
+      <c r="B86" s="56" t="n">
         <v>296028</v>
       </c>
-      <c r="C86" s="14" t="n">
+      <c r="C86" s="56" t="n">
         <v>15695</v>
       </c>
-      <c r="D86" s="14" t="n">
+      <c r="D86" s="56" t="n">
         <v>12275</v>
       </c>
-      <c r="E86" s="14" t="n">
+      <c r="E86" s="56" t="n">
         <v>19707</v>
       </c>
-      <c r="F86" s="14" t="n">
+      <c r="F86" s="56" t="n">
         <v>15989</v>
       </c>
       <c r="G86" s="14">
@@ -3262,24 +3114,22 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="43" t="inlineStr">
-        <is>
-          <t>03/30/2026</t>
-        </is>
-      </c>
-      <c r="B87" s="14" t="n">
+      <c r="A87" s="43" t="n">
+        <v>46111</v>
+      </c>
+      <c r="B87" s="56" t="n">
         <v>299746</v>
       </c>
-      <c r="C87" s="14" t="n">
+      <c r="C87" s="56" t="n">
         <v>16339</v>
       </c>
-      <c r="D87" s="14" t="n">
+      <c r="D87" s="56" t="n">
         <v>14656</v>
       </c>
-      <c r="E87" s="14" t="n">
+      <c r="E87" s="56" t="n">
         <v>18889</v>
       </c>
-      <c r="F87" s="14" t="n">
+      <c r="F87" s="56" t="n">
         <v>17836</v>
       </c>
       <c r="G87" s="14">
@@ -3292,24 +3142,22 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="43" t="inlineStr">
-        <is>
-          <t>04/06/2026</t>
-        </is>
-      </c>
-      <c r="B88" s="14" t="n">
+      <c r="A88" s="43" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B88" s="56" t="n">
         <v>300799</v>
       </c>
-      <c r="C88" s="14" t="n">
+      <c r="C88" s="56" t="n">
         <v>16175</v>
       </c>
-      <c r="D88" s="14" t="n">
+      <c r="D88" s="56" t="n">
         <v>14481</v>
       </c>
-      <c r="E88" s="14" t="n">
+      <c r="E88" s="56" t="n">
         <v>18562</v>
       </c>
-      <c r="F88" s="14" t="n">
+      <c r="F88" s="56" t="n">
         <v>17203</v>
       </c>
       <c r="G88" s="14">
@@ -3322,24 +3170,22 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="43" t="inlineStr">
-        <is>
-          <t>04/13/2026</t>
-        </is>
-      </c>
-      <c r="B89" s="14" t="n">
+      <c r="A89" s="43" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B89" s="56" t="n">
         <v>302158</v>
       </c>
-      <c r="C89" s="14" t="n">
+      <c r="C89" s="56" t="n">
         <v>18411</v>
       </c>
-      <c r="D89" s="14" t="n">
+      <c r="D89" s="56" t="n">
         <v>14251</v>
       </c>
-      <c r="E89" s="14" t="n">
+      <c r="E89" s="56" t="n">
         <v>20631</v>
       </c>
-      <c r="F89" s="14" t="n">
+      <c r="F89" s="56" t="n">
         <v>16627</v>
       </c>
       <c r="G89" s="14">
@@ -3352,24 +3198,22 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="43" t="inlineStr">
-        <is>
-          <t>04/20/2026</t>
-        </is>
-      </c>
-      <c r="B90" s="14" t="n">
+      <c r="A90" s="43" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B90" s="56" t="n">
         <v>306162</v>
       </c>
-      <c r="C90" s="14" t="n">
+      <c r="C90" s="56" t="n">
         <v>15925</v>
       </c>
-      <c r="D90" s="14" t="n">
+      <c r="D90" s="56" t="n">
         <v>14204</v>
       </c>
-      <c r="E90" s="14" t="n">
+      <c r="E90" s="56" t="n">
         <v>18787</v>
       </c>
-      <c r="F90" s="14" t="n">
+      <c r="F90" s="56" t="n">
         <v>18196</v>
       </c>
       <c r="G90" s="14">
@@ -3382,24 +3226,22 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="43" t="inlineStr">
-        <is>
-          <t>04/27/2026</t>
-        </is>
-      </c>
-      <c r="B91" s="14" t="n">
+      <c r="A91" s="43" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B91" s="56" t="n">
         <v>306753</v>
       </c>
-      <c r="C91" s="14" t="n">
+      <c r="C91" s="56" t="n">
         <v>17666</v>
       </c>
-      <c r="D91" s="14" t="n">
+      <c r="D91" s="56" t="n">
         <v>14942</v>
       </c>
-      <c r="E91" s="14" t="n">
+      <c r="E91" s="56" t="n">
         <v>20748</v>
       </c>
-      <c r="F91" s="14" t="n">
+      <c r="F91" s="56" t="n">
         <v>18306</v>
       </c>
       <c r="G91" s="14">
@@ -3412,24 +3254,22 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="43" t="inlineStr">
-        <is>
-          <t>05/04/2026</t>
-        </is>
-      </c>
-      <c r="B92" s="14" t="n">
+      <c r="A92" s="43" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B92" s="56" t="n">
         <v>309195</v>
       </c>
-      <c r="C92" s="14" t="n">
+      <c r="C92" s="56" t="n">
         <v>16743</v>
       </c>
-      <c r="D92" s="14" t="n">
+      <c r="D92" s="56" t="n">
         <v>12998</v>
       </c>
-      <c r="E92" s="14" t="n">
+      <c r="E92" s="56" t="n">
         <v>18809</v>
       </c>
-      <c r="F92" s="14" t="n">
+      <c r="F92" s="56" t="n">
         <v>16710</v>
       </c>
       <c r="G92" s="14">
@@ -3442,24 +3282,22 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="43" t="inlineStr">
-        <is>
-          <t>05/11/2026</t>
-        </is>
-      </c>
-      <c r="B93" s="14" t="n">
+      <c r="A93" s="43" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B93" s="56" t="n">
         <v>311294</v>
       </c>
-      <c r="C93" s="14" t="n">
+      <c r="C93" s="56" t="n">
         <v>16223</v>
       </c>
-      <c r="D93" s="14" t="n">
+      <c r="D93" s="56" t="n">
         <v>15796</v>
       </c>
-      <c r="E93" s="14" t="n">
+      <c r="E93" s="56" t="n">
         <v>20495</v>
       </c>
-      <c r="F93" s="14" t="n">
+      <c r="F93" s="56" t="n">
         <v>17431</v>
       </c>
       <c r="G93" s="14">
@@ -3472,24 +3310,22 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="43" t="inlineStr">
-        <is>
-          <t>05/18/2026</t>
-        </is>
-      </c>
-      <c r="B94" s="14" t="n">
+      <c r="A94" s="43" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B94" s="56" t="n">
         <v>314358</v>
       </c>
-      <c r="C94" s="14" t="n">
+      <c r="C94" s="56" t="n">
         <v>15806</v>
       </c>
-      <c r="D94" s="14" t="n">
+      <c r="D94" s="56" t="n">
         <v>16216</v>
       </c>
-      <c r="E94" s="14" t="n">
+      <c r="E94" s="56" t="n">
         <v>19423</v>
       </c>
-      <c r="F94" s="14" t="n">
+      <c r="F94" s="56" t="n">
         <v>18639</v>
       </c>
       <c r="G94" s="14">
@@ -3783,6 +3619,7 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="21.95" customHeight="1">
       <c r="A12" s="38" t="inlineStr">
         <is>

</xml_diff>